<commit_message>
补上Allen BIT 23 linfeng github page
</commit_message>
<xml_diff>
--- a/collected-data.xlsx
+++ b/collected-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-26.04\home\leo\OS-Agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DFC056-8FF7-445B-8CE6-484A5082A82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD397F4-2E78-442B-A31A-83A72B33B1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3083" uniqueCount="952">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3086" uniqueCount="954">
   <si>
     <t>年份</t>
   </si>
@@ -2813,10 +2813,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://gitlab.eduxiji.net/hzc1998/oskernel2021-xbook2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://gitlab.eduxiji.net/lightenos/oskernel2025-lightenos</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2829,10 +2825,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>已私密/删库</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://gitlab.eduxiji.net/potato-kernal/cy-os</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2926,6 +2918,22 @@
   </si>
   <si>
     <t>失效</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://gitee.com/hzc1998/xbook2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gitee版最新，github版： https://github.com/hzcx998/xbook2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://gitlab.eduxiji.net/os-contest-2021-kernel-final-scene/potato-kernal-cy-os</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">github版  https://github.com/Godones/Alien  </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3901,7 +3909,7 @@
         <v>17</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>63</v>
@@ -3910,7 +3918,9 @@
       <c r="K16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L16" s="3"/>
+      <c r="L16" s="3" t="s">
+        <v>953</v>
+      </c>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
@@ -4014,7 +4024,7 @@
         <v>77</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>79</v>
@@ -4187,19 +4197,19 @@
         <v>17</v>
       </c>
       <c r="H24" s="1" t="s">
+        <v>933</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>934</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>935</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>926</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>936</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>926</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>937</v>
       </c>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
@@ -4839,16 +4849,16 @@
         <v>19</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>17</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
@@ -4875,7 +4885,7 @@
         <v>17</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>19</v>
@@ -6584,25 +6594,25 @@
         <v>314</v>
       </c>
       <c r="E90" s="3" t="s">
+        <v>940</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>941</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H90" s="1" t="s">
         <v>942</v>
       </c>
-      <c r="F90" s="1" t="s">
+      <c r="I90" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="J90" s="1" t="s">
         <v>943</v>
       </c>
-      <c r="G90" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H90" s="1" t="s">
-        <v>944</v>
-      </c>
-      <c r="I90" s="3" t="s">
-        <v>926</v>
-      </c>
-      <c r="J90" s="1" t="s">
-        <v>945</v>
-      </c>
       <c r="K90" s="3" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="L90" s="3"/>
       <c r="M90" s="3"/>
@@ -6773,19 +6783,19 @@
         <v>335</v>
       </c>
       <c r="F95" s="1" t="s">
+        <v>944</v>
+      </c>
+      <c r="G95" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H95" s="1" t="s">
         <v>946</v>
       </c>
-      <c r="G95" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H95" s="1" t="s">
-        <v>948</v>
-      </c>
       <c r="I95" s="3" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="K95" s="3" t="s">
         <v>19</v>
@@ -7105,16 +7115,16 @@
         <v>17</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="I104" s="3" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="J104" s="1" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="K104" s="3" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="L104" s="3"/>
       <c r="M104" s="3"/>
@@ -7764,7 +7774,7 @@
         <v>431</v>
       </c>
       <c r="I122" s="3" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="J122" s="1" t="s">
         <v>922</v>
@@ -8773,7 +8783,7 @@
         <v>17</v>
       </c>
       <c r="J150" s="1" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="K150" s="3" t="s">
         <v>19</v>
@@ -8985,10 +8995,10 @@
         <v>19</v>
       </c>
       <c r="H156" s="1" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="I156" s="3" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="J156" s="3" t="s">
         <v>543</v>
@@ -9127,14 +9137,16 @@
         <v>17</v>
       </c>
       <c r="H160" s="1" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="I160" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="J160" s="3"/>
+      <c r="J160" s="1" t="s">
+        <v>952</v>
+      </c>
       <c r="K160" s="3" t="s">
-        <v>17</v>
+        <v>925</v>
       </c>
       <c r="L160" s="3"/>
       <c r="M160" s="3"/>
@@ -9339,13 +9351,13 @@
         <v>17</v>
       </c>
       <c r="H166" s="1" t="s">
+        <v>923</v>
+      </c>
+      <c r="I166" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="J166" s="1" t="s">
         <v>924</v>
-      </c>
-      <c r="I166" s="3" t="s">
-        <v>926</v>
-      </c>
-      <c r="J166" s="1" t="s">
-        <v>925</v>
       </c>
       <c r="K166" s="3" t="s">
         <v>19</v>
@@ -9375,16 +9387,18 @@
         <v>17</v>
       </c>
       <c r="H167" s="1" t="s">
-        <v>923</v>
+        <v>950</v>
       </c>
       <c r="I167" s="3" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="J167" s="3"/>
       <c r="K167" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L167" s="3"/>
+      <c r="L167" s="3" t="s">
+        <v>951</v>
+      </c>
       <c r="M167" s="3"/>
       <c r="N167" s="3"/>
     </row>
@@ -15115,6 +15129,7 @@
     <hyperlink ref="J95" r:id="rId122" xr:uid="{88D346BF-DD10-4CE7-A12D-07F3955A5105}"/>
     <hyperlink ref="H95" r:id="rId123" xr:uid="{C4025397-2E5E-4A44-9264-51E3F5D4E892}"/>
     <hyperlink ref="H104" r:id="rId124" xr:uid="{C40B8DDE-14F9-420E-AAB9-72C840751240}"/>
+    <hyperlink ref="J160" r:id="rId125" xr:uid="{519864A7-D732-4BDC-9E57-FD28948FFEE2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>